<commit_message>
Update OCR label generator and QR payload
</commit_message>
<xml_diff>
--- a/data/scans.xlsx
+++ b/data/scans.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N311"/>
+  <dimension ref="A1:N314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23369,6 +23369,263 @@
       <c r="M311" t="inlineStr"/>
       <c r="N311" t="inlineStr"/>
     </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-03-14 06:32:57</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>KEMET</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>NUM8ER</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>45239701</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>2542</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>paddleocr</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>7.82s</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>P
+P PART NUM8ER:KEMCO805S104KSRA
+'
+Q QUANTITY2S00
+CAPACITOR
+ROHS-PRC
+T
+−
+.100UF 50V
+10%
+DATE CODE :2542
+1T LOT:254270641
+C OF O MEXICO
+046
+45239701
+KEMET P/N CO8OSS104KSRAC7800
+KEMET
+MIL P/N
+A YAGEO COMPONY
+C
+7</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>53de29547c962802e57a5cb16ec745c5b3811a4d7480e23f38dfacbdb088a002</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>254270641</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>CAPACITOR</t>
+        </is>
+      </c>
+      <c r="M312" t="n">
+        <v>1.000001000183201e+17</v>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>185101626</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-03-14 06:33:45</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>KEMET</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>KEMCO8OSS104KSRA</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>45239701</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>2542</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>paddleocr</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>7.57s</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>U
+4
+P PART NUMBER:KEMCO8OSS104KSRA
+Q QUANTITY 2SOO
+CAPACITOR
+ROHS-PRC
+.100UF SOV
+10%
+DATE CODE :2542
+1T LOT :254270641
+C OF O MEXICO
+T
+5":415 (11]
+UAIA
+45239701
+KEMET P/N CO8OSS104KSRAC7800
+KEMET
+MIL P/N
+• YAGTO COMPARY
+A
+Y
+R</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>12ff412711e55208f1087c07c64b8bfc2ab78a93e3bb43463c7d24f2112eeb17</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>254270641</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>CAPACITOR</t>
+        </is>
+      </c>
+      <c r="M313" t="n">
+        <v>1.000001000183201e+17</v>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>185101626</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-03-14 06:33:53</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>KEMET</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>KEMC0805S104KSRA</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr"/>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>paddleocr</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>6.66s</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>!
+7
+P PART NUMBER:KEMCO805S104KSRA
+Q QUANTITY 2500
+CAPACITOR
+ROHS-PRC
+.100UF 50V
+10%
+DATE CODE :2S42
+1T LOT :254270641
+C OF O MEXICO
+SPL4IE
+45239701
+KEMET P/N CO8OSS104KSRAC7800
+KEMET
+MIL P/N
+O YAGEO COMPORTY</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>5d1f6dfc5634fe5728183691d2412682bee342086609b31d362484d08ac32de6</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>254270641</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>CAPACITOR</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>100000100018320103</t>
+        </is>
+      </c>
+      <c r="N314" t="inlineStr">
+        <is>
+          <t>185101626</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>